<commit_message>
updates for 2024 q4 partial
</commit_message>
<xml_diff>
--- a/pie_community_logos.xlsx
+++ b/pie_community_logos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vwallace.secure\Documents\Git Repos\PIE-Logos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BGDatabaseService\Documents\PIE-Logos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1089C09-8671-498F-9413-6508E88552F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C66E54E-AB7E-4312-8200-6021741C5405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21000" xr2:uid="{570DFFD5-5DC0-480E-9EEE-DC9F928AA597}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="140">
   <si>
     <t>state_name</t>
   </si>
@@ -299,9 +299,6 @@
     <t>Menomonie</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Minnesota/Bloomington.png</t>
-  </si>
-  <si>
     <t>Adams County</t>
   </si>
   <si>
@@ -332,7 +329,133 @@
     <t>Sterling Ranch Update</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado</t>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/adams%20county.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/arapahoe%20county.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/arvada.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/aurora.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/Boulder%20County.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/boulder.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/broomfield.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/centennial.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/central%20city%20colorado.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/Denver%20Zoo.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/DMNS.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/denver.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/edgewater.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/englewood.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/erie.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/fort%20collins%20utilities.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/Frisco.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/garfield%20county.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/grand%20county.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/greeley.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/jeffco.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/jefferson.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/lafayette.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/Lake%20County.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/lakewood.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/littleton.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/lone%20tree.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/longmont.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/Louisville.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/minturn.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/nederland.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/northglenn.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/pueblo%20county.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/Salida.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/sterling%20ranch.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/summit%20county.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/superior.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/thornton.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/westminster.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/wheatridge.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado/windsor.png</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Minnesota/Bloomington.png/</t>
   </si>
 </sst>
 </file>
@@ -739,10 +862,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -764,7 +887,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -775,7 +898,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -783,10 +906,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -794,10 +917,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -808,7 +931,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -819,7 +942,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -827,10 +950,10 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -841,7 +964,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -852,7 +975,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -860,10 +983,10 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -874,7 +997,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
@@ -882,10 +1005,10 @@
         <v>3</v>
       </c>
       <c r="B15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -896,7 +1019,7 @@
         <v>12</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
@@ -907,7 +1030,7 @@
         <v>13</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
@@ -918,7 +1041,7 @@
         <v>14</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -929,7 +1052,7 @@
         <v>15</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -940,7 +1063,7 @@
         <v>16</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -948,10 +1071,10 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -962,7 +1085,7 @@
         <v>17</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -973,7 +1096,7 @@
         <v>18</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -984,7 +1107,7 @@
         <v>19</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
@@ -995,7 +1118,7 @@
         <v>20</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
@@ -1006,7 +1129,7 @@
         <v>21</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
@@ -1017,7 +1140,7 @@
         <v>22</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>98</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
@@ -1028,7 +1151,7 @@
         <v>23</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -1039,7 +1162,7 @@
         <v>24</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
@@ -1050,7 +1173,7 @@
         <v>25</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
@@ -1061,7 +1184,7 @@
         <v>26</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
@@ -1072,7 +1195,7 @@
         <v>27</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.35">
@@ -1083,7 +1206,7 @@
         <v>28</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>98</v>
+        <v>124</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.35">
@@ -1094,7 +1217,7 @@
         <v>29</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>98</v>
+        <v>125</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.35">
@@ -1105,7 +1228,7 @@
         <v>30</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>98</v>
+        <v>126</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.35">
@@ -1116,7 +1239,7 @@
         <v>31</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.35">
@@ -1127,7 +1250,7 @@
         <v>32</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.35">
@@ -1138,7 +1261,7 @@
         <v>33</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.35">
@@ -1149,7 +1272,7 @@
         <v>34</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.35">
@@ -1160,7 +1283,7 @@
         <v>35</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>98</v>
+        <v>130</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.35">
@@ -1171,7 +1294,7 @@
         <v>36</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.35">
@@ -1179,10 +1302,10 @@
         <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.35">
@@ -1190,10 +1313,10 @@
         <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.35">
@@ -1204,7 +1327,7 @@
         <v>37</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>98</v>
+        <v>132</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.35">
@@ -1212,10 +1335,10 @@
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.35">
@@ -1226,7 +1349,7 @@
         <v>38</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.35">
@@ -1237,7 +1360,7 @@
         <v>39</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>98</v>
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.35">
@@ -1248,7 +1371,7 @@
         <v>40</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>98</v>
+        <v>135</v>
       </c>
       <c r="S48" s="1"/>
     </row>
@@ -1260,7 +1383,7 @@
         <v>41</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>98</v>
+        <v>136</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
@@ -1271,7 +1394,7 @@
         <v>42</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
@@ -1282,7 +1405,7 @@
         <v>43</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>98</v>
+        <v>138</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
@@ -1293,7 +1416,7 @@
         <v>45</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>87</v>
+        <v>139</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
@@ -1618,9 +1741,9 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C52" r:id="rId1" xr:uid="{C38D9350-DE2A-4E63-9A1C-3C89746D249E}"/>
-    <hyperlink ref="C2" r:id="rId2" xr:uid="{715CEFF7-4C4A-457A-9C38-A4888F1259FB}"/>
-    <hyperlink ref="C3:C51" r:id="rId3" display="https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado" xr:uid="{AB4769A4-453C-4910-9BBB-3BB95B3E17F6}"/>
+    <hyperlink ref="C3:C51" r:id="rId1" display="https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado" xr:uid="{AB4769A4-453C-4910-9BBB-3BB95B3E17F6}"/>
+    <hyperlink ref="C2" r:id="rId2" display="https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Colorado" xr:uid="{715CEFF7-4C4A-457A-9C38-A4888F1259FB}"/>
+    <hyperlink ref="C52" r:id="rId3" display="https://raw.githubusercontent.com/Brendle-Group/PIE-Logos/refs/heads/main/Minnesota/Bloomington.png" xr:uid="{C38D9350-DE2A-4E63-9A1C-3C89746D249E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>